<commit_message>
add test benefit others
</commit_message>
<xml_diff>
--- a/e2e/data/test-data.xlsx
+++ b/e2e/data/test-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Telkomcel\test\e2e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2215DCA8-88E5-429B-9464-37D5A2A5449B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6DD4C8E-1217-4D95-99DF-2B8EF235F34F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="225" yWindow="2640" windowWidth="23775" windowHeight="10140" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DaftarGaji" sheetId="1" r:id="rId1"/>
@@ -18,16 +18,16 @@
     <sheet name="Overtime" sheetId="3" r:id="rId3"/>
     <sheet name="Pulsa" sheetId="4" r:id="rId4"/>
     <sheet name="Medical" sheetId="5" r:id="rId5"/>
-    <sheet name="Other" sheetId="6" r:id="rId6"/>
-    <sheet name="OtherProrate" sheetId="7" r:id="rId7"/>
-    <sheet name="Prorate" sheetId="8" r:id="rId8"/>
+    <sheet name="OtherProrate" sheetId="6" r:id="rId6"/>
+    <sheet name="Prorate" sheetId="7" r:id="rId7"/>
+    <sheet name="Benefit Others" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="105">
   <si>
     <t>id</t>
   </si>
@@ -284,21 +284,12 @@
     <t>2</t>
   </si>
   <si>
+    <t>tarif</t>
+  </si>
+  <si>
     <t>payment</t>
   </si>
   <si>
-    <t>2026-08</t>
-  </si>
-  <si>
-    <t>THR</t>
-  </si>
-  <si>
-    <t>Bonus</t>
-  </si>
-  <si>
-    <t>tarif</t>
-  </si>
-  <si>
     <t>remarks</t>
   </si>
   <si>
@@ -336,6 +327,21 @@
   </si>
   <si>
     <t>2026-01-31</t>
+  </si>
+  <si>
+    <t>salary</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>2026-01-12</t>
+  </si>
+  <si>
+    <t>Catatan January rimbun siburian</t>
+  </si>
+  <si>
+    <t>Catatan January Celia Maria Rego</t>
   </si>
 </sst>
 </file>
@@ -713,9 +719,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -747,7 +753,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -779,7 +785,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -811,7 +817,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -843,7 +849,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -875,7 +881,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -907,7 +913,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -939,7 +945,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -971,7 +977,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1003,7 +1009,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1035,7 +1041,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1067,7 +1073,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1099,7 +1105,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1133,6 +1139,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="A1:J13" numberStoredAsText="1"/>
   </ignoredErrors>
@@ -1142,9 +1149,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1170,7 +1177,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1196,7 +1203,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1222,7 +1229,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1248,7 +1255,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1274,7 +1281,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1300,7 +1307,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1326,7 +1333,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1352,7 +1359,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1389,9 +1396,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1420,7 +1427,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1449,7 +1456,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1478,7 +1485,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1507,7 +1514,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1536,7 +1543,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1565,7 +1572,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>7</v>
       </c>
@@ -1594,7 +1601,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>8</v>
       </c>
@@ -1623,7 +1630,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9</v>
       </c>
@@ -1663,9 +1670,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1685,7 +1692,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1705,7 +1712,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1725,7 +1732,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1745,7 +1752,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1765,7 +1772,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1785,7 +1792,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1805,7 +1812,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1836,9 +1843,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1858,7 +1865,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1878,7 +1885,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1898,7 +1905,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1918,7 +1925,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1938,7 +1945,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1958,7 +1965,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1978,7 +1985,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1998,7 +2005,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2018,7 +2025,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2038,7 +2045,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2058,7 +2065,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2078,7 +2085,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2098,7 +2105,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2118,7 +2125,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2138,7 +2145,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2168,10 +2175,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2188,13 +2195,16 @@
         <v>85</v>
       </c>
       <c r="F1" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="G1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+      <c r="H1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2205,19 +2215,22 @@
         <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F2" t="s">
-        <v>55</v>
+        <v>54</v>
+      </c>
+      <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="F2">
+        <v>2.2999999999999998</v>
       </c>
       <c r="G2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+      <c r="H2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2228,94 +2241,6 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3" t="s">
-        <v>88</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:G3" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" t="s">
-        <v>89</v>
-      </c>
-      <c r="F1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E2">
-        <v>10</v>
-      </c>
-      <c r="F2">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="G2" t="s">
-        <v>91</v>
-      </c>
-      <c r="H2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
         <v>54</v>
       </c>
       <c r="E3">
@@ -2325,10 +2250,10 @@
         <v>2.5</v>
       </c>
       <c r="G3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -2339,12 +2264,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2355,28 +2280,28 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E1" t="s">
         <v>50</v>
       </c>
       <c r="F1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H1" t="s">
+        <v>94</v>
+      </c>
+      <c r="I1" t="s">
         <v>95</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>96</v>
       </c>
-      <c r="H1" t="s">
-        <v>97</v>
-      </c>
-      <c r="I1" t="s">
-        <v>98</v>
-      </c>
-      <c r="J1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2387,7 +2312,7 @@
         <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E2" t="s">
         <v>54</v>
@@ -2396,19 +2321,19 @@
         <v>31</v>
       </c>
       <c r="G2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I2" t="s">
         <v>72</v>
       </c>
       <c r="J2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2419,7 +2344,7 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E3" t="s">
         <v>54</v>
@@ -2428,16 +2353,16 @@
         <v>30</v>
       </c>
       <c r="G3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I3" t="s">
         <v>72</v>
       </c>
       <c r="J3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2446,4 +2371,101 @@
     <ignoredError sqref="A1:J3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2">
+        <v>500</v>
+      </c>
+      <c r="F2">
+        <v>0.25</v>
+      </c>
+      <c r="G2" t="s">
+        <v>102</v>
+      </c>
+      <c r="H2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3">
+        <v>300.23</v>
+      </c>
+      <c r="F3">
+        <v>0.25</v>
+      </c>
+      <c r="G3" t="s">
+        <v>102</v>
+      </c>
+      <c r="H3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:H2" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>